<commit_message>
Design update, improved visual presentation.
</commit_message>
<xml_diff>
--- a/output/remote_jobs.xlsx
+++ b/output/remote_jobs.xlsx
@@ -479,7 +479,11 @@
           <t>accountant, support, accounting, payroll, financial, sales, health, healthcare, non tech</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F2" t="inlineStr">
         <is>
           <t>2026-03-05T19:00:05+00:00</t>
@@ -517,7 +521,11 @@
           <t>python, game, technical, support, code, math, node, lead</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F3" t="inlineStr">
         <is>
           <t>2026-03-09T22:00:13+00:00</t>
@@ -555,7 +563,11 @@
           <t>game, design, designer, mobile, strategy, content, senior, junior, digital nomad</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F4" t="inlineStr">
         <is>
           <t>2026-02-28T21:00:14+00:00</t>
@@ -593,7 +605,11 @@
           <t>director, students, training, support, software</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F5" t="inlineStr">
         <is>
           <t>2026-03-10T06:00:23+00:00</t>
@@ -631,7 +647,11 @@
           <t>architect, design, security, training, technical, growth, serverless, cloud, management, lead, junior, health, engineering, digital nomad</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F6" t="inlineStr">
         <is>
           <t>2026-03-03T21:00:19+00:00</t>
@@ -669,7 +689,11 @@
           <t>design, security, training, architect, technical, support, cloud, node, management, operational, health, engineer, digital nomad</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F7" t="inlineStr">
         <is>
           <t>2026-03-07T20:00:08+00:00</t>
@@ -707,7 +731,11 @@
           <t>design, crypto, security, support, financial, investment, api, lead, operations, operational, digital nomad</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F8" t="inlineStr">
         <is>
           <t>2026-03-09T07:00:07+00:00</t>
@@ -745,7 +773,11 @@
           <t>analyst, crypto, training, support, financial, investment, fintech, api, operations, sales, non tech</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F9" t="inlineStr">
         <is>
           <t>2026-03-05T11:00:07+00:00</t>
@@ -825,7 +857,11 @@
           <t>manager, technical, software, cloud, operational, engineering</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F11" t="inlineStr">
         <is>
           <t>2026-03-07T13:00:12+00:00</t>
@@ -863,7 +899,11 @@
           <t>design, game, technical, developer, animator, animation, content, senior, digital nomad</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F12" t="inlineStr">
         <is>
           <t>2026-03-03T21:00:06+00:00</t>
@@ -901,7 +941,11 @@
           <t>assistant, design, support, admin, content, sales, executive, full-time, digital nomad</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F13" t="inlineStr">
         <is>
           <t>2026-03-03T07:00:02+00:00</t>
@@ -939,7 +983,11 @@
           <t>support, operational, analytics, engineering</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F14" t="inlineStr">
         <is>
           <t>2026-03-07T00:00:35+00:00</t>
@@ -977,7 +1025,11 @@
           <t>developer, back-end, python, reliability, backend, ecommerce, e-commerce, digital nomad</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F15" t="inlineStr">
         <is>
           <t>2026-03-06T02:00:12+00:00</t>
@@ -1057,7 +1109,11 @@
           <t>design, designer, growth, web, marketing, go, health, digital nomad</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F17" t="inlineStr">
         <is>
           <t>2026-03-10T10:00:06+00:00</t>
@@ -1097,7 +1153,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>6000</t>
+          <t>6000-0</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1137,7 +1193,11 @@
           <t>design, system, technical, support, growth, director, lead, senior, engineer, engineering, digital nomad</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F19" t="inlineStr">
         <is>
           <t>2026-03-05T23:00:14+00:00</t>
@@ -1175,7 +1235,11 @@
           <t>manager, web3, security, technical, support, travel, lead, sales, full-time</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr"/>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F20" t="inlineStr">
         <is>
           <t>2026-03-05T15:00:04+00:00</t>
@@ -1213,7 +1277,11 @@
           <t>teach, technical, support, code, engineer, engineering</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr"/>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F21" t="inlineStr">
         <is>
           <t>2026-03-03T17:00:17+00:00</t>
@@ -1251,7 +1319,11 @@
           <t>design, ansible, security, python, training, support, growth, code, voice, devops, education, banking, mobile, management, senior, sales, go, health, recruiting, engineer, engineering, recruitment, linux, e-commerce, digital nomad</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr"/>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F22" t="inlineStr">
         <is>
           <t>2026-03-07T00:01:33+00:00</t>
@@ -1289,7 +1361,11 @@
           <t>manager, design, saas, training, support, growth, director, voice, education, banking, mobile, strategy, lead, senior, operations, marketing, sales, go, health, recruiting, recruitment, executive, digital nomad</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr"/>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F23" t="inlineStr">
         <is>
           <t>2026-03-04T00:01:20+00:00</t>
@@ -1327,7 +1403,11 @@
           <t>security, software, growth, video, analytics</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr"/>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F24" t="inlineStr">
         <is>
           <t>2026-03-04T00:01:42+00:00</t>
@@ -1365,7 +1445,11 @@
           <t>design, saas, technical, support, growth, strategy, management, operations, operational, digital nomad</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr"/>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F25" t="inlineStr">
         <is>
           <t>2026-03-09T17:00:06+00:00</t>
@@ -1403,7 +1487,11 @@
           <t>manager, crypto, cryptocurrency, api, operational, marketing, sales</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr"/>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F26" t="inlineStr">
         <is>
           <t>2026-03-03T18:00:01+00:00</t>
@@ -1441,7 +1529,11 @@
           <t>analyst, embedded, security, training, consultancy, management, senior, executive</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr"/>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F27" t="inlineStr">
         <is>
           <t>2026-03-04T00:00:42+00:00</t>
@@ -1479,7 +1571,11 @@
           <t>react, software, design, jira, front-end, back-end, security, training, test, code, web, javascript, html, senior, engineer, engineering, digital nomad</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr"/>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F28" t="inlineStr">
         <is>
           <t>2026-03-05T16:00:14+00:00</t>
@@ -1517,7 +1613,11 @@
           <t>support, software, devops, cloud, lead, content, reliability, engineer, engineering</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr"/>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F29" t="inlineStr">
         <is>
           <t>2026-03-07T20:00:19+00:00</t>
@@ -1555,7 +1655,11 @@
           <t>financial, fintech, banking, senior, engineer</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr"/>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F30" t="inlineStr">
         <is>
           <t>2026-03-04T08:00:21+00:00</t>
@@ -1635,7 +1739,11 @@
           <t>senior, sales, engineer</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr"/>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F32" t="inlineStr">
         <is>
           <t>2026-03-10T00:01:04+00:00</t>
@@ -1673,7 +1781,11 @@
           <t>vfx, technical, lead, engineering</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr"/>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F33" t="inlineStr">
         <is>
           <t>2026-03-03T22:00:12+00:00</t>
@@ -1711,7 +1823,11 @@
           <t>unity, designer, senior</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr"/>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F34" t="inlineStr">
         <is>
           <t>2026-03-03T22:00:26+00:00</t>
@@ -1749,7 +1865,11 @@
           <t>growth, design, frontend, architect, technical, web, mobile, leader, lead, executive, digital nomad</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr"/>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F35" t="inlineStr">
         <is>
           <t>2026-03-04T00:01:31+00:00</t>
@@ -1787,7 +1907,11 @@
           <t>manager, system, technical, software, ui, code, engineering</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr"/>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F36" t="inlineStr">
         <is>
           <t>2026-03-03T00:01:09+00:00</t>
@@ -1825,7 +1949,11 @@
           <t>security, design, api, engineer, engineering, digital nomad</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr"/>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F37" t="inlineStr">
         <is>
           <t>2026-03-09T08:00:05+00:00</t>
@@ -1863,7 +1991,11 @@
           <t>support, software, senior, engineer, engineering</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr"/>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F38" t="inlineStr">
         <is>
           <t>2026-03-03T16:00:17+00:00</t>
@@ -1901,7 +2033,11 @@
           <t>support, financial, finance, fintech, strategy, operations, non tech</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr"/>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F39" t="inlineStr">
         <is>
           <t>2026-03-04T00:00:08+00:00</t>
@@ -1939,7 +2075,11 @@
           <t>manager, hr, training, growth, management, lead, senior, operations, reliability</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr"/>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F40" t="inlineStr">
         <is>
           <t>2026-03-03T00:00:53+00:00</t>
@@ -1977,7 +2117,11 @@
           <t>python, django, software, design, saas, security, full-stack, technical, developer, testing, code, devops, cloud, git, postgresql, senior, operations, engineer, digital nomad</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr"/>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F41" t="inlineStr">
         <is>
           <t>2026-03-09T18:00:23+00:00</t>
@@ -2015,7 +2159,11 @@
           <t>web3, cryptocurrency, voice, lead, content, operations, executive</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr"/>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F42" t="inlineStr">
         <is>
           <t>2026-03-09T12:00:02+00:00</t>
@@ -2053,7 +2201,11 @@
           <t>salesforce, technical, support, administrator, management, reliability, health</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr"/>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F43" t="inlineStr">
         <is>
           <t>2026-03-03T18:00:12+00:00</t>
@@ -2091,7 +2243,11 @@
           <t>system, teaching, students, technical</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr"/>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F44" t="inlineStr">
         <is>
           <t>2026-03-10T00:01:14+00:00</t>
@@ -2129,7 +2285,11 @@
           <t>analyst, support, testing, leader, senior, health, healthcare, non tech</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr"/>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F45" t="inlineStr">
         <is>
           <t>2026-03-10T00:00:49+00:00</t>
@@ -2167,7 +2327,11 @@
           <t>design, lead, digital nomad</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr"/>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F46" t="inlineStr">
         <is>
           <t>2026-03-10T00:00:18+00:00</t>
@@ -2205,7 +2369,11 @@
           <t>accountant, saas, manager, accounting, financial, go</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr"/>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F47" t="inlineStr">
         <is>
           <t>2026-03-05T20:00:07+00:00</t>
@@ -2243,7 +2411,11 @@
           <t>training, support, education, admin, management, content, non tech</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr"/>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F48" t="inlineStr">
         <is>
           <t>2026-03-09T08:00:03+00:00</t>
@@ -2277,7 +2449,11 @@
         </is>
       </c>
       <c r="D49" t="inlineStr"/>
-      <c r="E49" t="inlineStr"/>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F49" t="inlineStr">
         <is>
           <t>2026-03-04T16:00:04+00:00</t>
@@ -2315,7 +2491,11 @@
           <t>analyst, support, financial, senior, analytics, health, non tech</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr"/>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F50" t="inlineStr">
         <is>
           <t>2026-03-07T00:00:56+00:00</t>
@@ -2353,7 +2533,11 @@
           <t>manager, design, system, architect, technical, support, growth, voice, lead, medical, health, engineering, digital nomad</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr"/>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F51" t="inlineStr">
         <is>
           <t>2026-03-07T00:00:08+00:00</t>
@@ -2391,7 +2575,11 @@
           <t>manager, design, saas, support, growth, financial, investment, investor, fintech, strategy, management, senior, operational, analytics, sales, reliability, engineering, digital nomad</t>
         </is>
       </c>
-      <c r="E52" t="inlineStr"/>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F52" t="inlineStr">
         <is>
           <t>2026-03-03T00:00:13+00:00</t>
@@ -2429,7 +2617,11 @@
           <t>design, full-stack, architect, testing, operational, engineer, engineering, digital nomad</t>
         </is>
       </c>
-      <c r="E53" t="inlineStr"/>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F53" t="inlineStr">
         <is>
           <t>2026-03-10T00:00:27+00:00</t>
@@ -2467,7 +2659,11 @@
           <t>manager, saas, security, technical, growth, voice, bank, management, lead, android, sales, recruitment, executive</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr"/>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F54" t="inlineStr">
         <is>
           <t>2026-03-03T08:00:20+00:00</t>
@@ -2505,7 +2701,11 @@
           <t>manager, copywriting, growth, strategy, management, content, junior</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr"/>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F55" t="inlineStr">
         <is>
           <t>2026-03-06T08:00:04+00:00</t>
@@ -2543,7 +2743,11 @@
           <t>full-stack, devops, financial, fintech, cloud, senior, engineer</t>
         </is>
       </c>
-      <c r="E56" t="inlineStr"/>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F56" t="inlineStr">
         <is>
           <t>2026-03-04T00:00:17+00:00</t>
@@ -2623,7 +2827,11 @@
           <t>system, security, software, devops, operations, operational, engineer, linux</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr"/>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F58" t="inlineStr">
         <is>
           <t>2026-03-04T17:00:05+00:00</t>
@@ -2661,7 +2869,11 @@
           <t>embedded, growth, analytics, engineer, engineering</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr"/>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F59" t="inlineStr">
         <is>
           <t>2026-03-03T16:00:07+00:00</t>
@@ -2699,7 +2911,11 @@
           <t>design, embedded, teach, students, designer, financial, banking, senior, internship, digital nomad</t>
         </is>
       </c>
-      <c r="E60" t="inlineStr"/>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F60" t="inlineStr">
         <is>
           <t>2026-03-03T12:00:05+00:00</t>
@@ -2737,7 +2953,11 @@
           <t>system, coordinator, support, management, operational, medical, health, healthcare</t>
         </is>
       </c>
-      <c r="E61" t="inlineStr"/>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F61" t="inlineStr">
         <is>
           <t>2026-03-07T00:00:20+00:00</t>
@@ -2775,7 +2995,11 @@
           <t>training, support, leader, content, health, non tech</t>
         </is>
       </c>
-      <c r="E62" t="inlineStr"/>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F62" t="inlineStr">
         <is>
           <t>2026-03-07T00:01:21+00:00</t>
@@ -2813,7 +3037,11 @@
           <t>game, design, designer, technical, lead, content, senior, digital nomad</t>
         </is>
       </c>
-      <c r="E63" t="inlineStr"/>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F63" t="inlineStr">
         <is>
           <t>2026-02-28T21:00:04+00:00</t>
@@ -2851,7 +3079,11 @@
           <t>manager, embedded, growth, director, senior, operational, medical, health</t>
         </is>
       </c>
-      <c r="E64" t="inlineStr"/>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F64" t="inlineStr">
         <is>
           <t>2026-03-10T00:00:42+00:00</t>
@@ -2889,7 +3121,11 @@
           <t>software, design, technical, leader, senior, medical, health, engineer, digital nomad</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr"/>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F65" t="inlineStr">
         <is>
           <t>2026-03-10T16:00:07+00:00</t>
@@ -2927,7 +3163,11 @@
           <t>director, training, consult, support, growth, travel, voice, financial, c, leader, strategy, management, lead, senior, marketing, sales, health, recruitment, executive, full-time</t>
         </is>
       </c>
-      <c r="E66" t="inlineStr"/>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F66" t="inlineStr">
         <is>
           <t>2026-03-10T00:00:56+00:00</t>
@@ -2965,7 +3205,11 @@
           <t>director, financial, management, sales</t>
         </is>
       </c>
-      <c r="E67" t="inlineStr"/>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F67" t="inlineStr">
         <is>
           <t>2026-03-03T08:00:13+00:00</t>
@@ -3003,7 +3247,11 @@
           <t>manager, financial, management, sales, non tech</t>
         </is>
       </c>
-      <c r="E68" t="inlineStr"/>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F68" t="inlineStr">
         <is>
           <t>2026-03-04T00:01:12+00:00</t>
@@ -3041,7 +3289,11 @@
           <t>director, saas, system, growth, leader, strategy, lead, sales, medical, health</t>
         </is>
       </c>
-      <c r="E69" t="inlineStr"/>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F69" t="inlineStr">
         <is>
           <t>2026-03-03T00:00:31+00:00</t>
@@ -3079,7 +3331,11 @@
           <t>technical, growth, strategy, lead, senior, health, engineering</t>
         </is>
       </c>
-      <c r="E70" t="inlineStr"/>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F70" t="inlineStr">
         <is>
           <t>2026-03-09T18:00:06+00:00</t>
@@ -3117,7 +3373,11 @@
           <t>software, react, front-end, technical, code, mobile, leader, health, healthcare, engineer, engineering</t>
         </is>
       </c>
-      <c r="E71" t="inlineStr"/>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F71" t="inlineStr">
         <is>
           <t>2026-03-04T00:00:29+00:00</t>
@@ -3155,7 +3415,11 @@
           <t>frontend, design, software, growth, web, management, engineer, backend, digital nomad</t>
         </is>
       </c>
-      <c r="E72" t="inlineStr"/>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F72" t="inlineStr">
         <is>
           <t>2026-03-09T09:00:04+00:00</t>
@@ -3193,7 +3457,11 @@
           <t>support, content</t>
         </is>
       </c>
-      <c r="E73" t="inlineStr"/>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F73" t="inlineStr">
         <is>
           <t>2026-03-03T18:00:40+00:00</t>
@@ -3231,7 +3499,11 @@
           <t>support, content</t>
         </is>
       </c>
-      <c r="E74" t="inlineStr"/>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F74" t="inlineStr">
         <is>
           <t>2026-03-03T18:00:21+00:00</t>
@@ -3269,7 +3541,11 @@
           <t>growth, marketing, analytics, sales, executive</t>
         </is>
       </c>
-      <c r="E75" t="inlineStr"/>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F75" t="inlineStr">
         <is>
           <t>2026-03-03T00:00:06+00:00</t>
@@ -3349,7 +3625,11 @@
           <t>training, technical, testing, test, code, travel, microsoft, senior, legal, health</t>
         </is>
       </c>
-      <c r="E77" t="inlineStr"/>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F77" t="inlineStr">
         <is>
           <t>2026-03-10T08:00:17+00:00</t>
@@ -3387,7 +3667,11 @@
           <t>full-stack, technical, support, growth, code, cloud, management, operational, sales, engineer, engineering</t>
         </is>
       </c>
-      <c r="E78" t="inlineStr"/>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F78" t="inlineStr">
         <is>
           <t>2026-03-06T07:00:06+00:00</t>
@@ -3425,7 +3709,11 @@
           <t>python, technical, support, financial, fintech, analytics, go, health, engineering</t>
         </is>
       </c>
-      <c r="E79" t="inlineStr"/>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F79" t="inlineStr">
         <is>
           <t>2026-03-10T08:00:11+00:00</t>
@@ -3463,7 +3751,11 @@
           <t>manager, support, operations, operational</t>
         </is>
       </c>
-      <c r="E80" t="inlineStr"/>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F80" t="inlineStr">
         <is>
           <t>2026-03-10T09:00:06+00:00</t>
@@ -3501,7 +3793,11 @@
           <t>system, technical, operations, operational</t>
         </is>
       </c>
-      <c r="E81" t="inlineStr"/>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F81" t="inlineStr">
         <is>
           <t>2026-03-03T08:00:03+00:00</t>
@@ -3539,7 +3835,11 @@
           <t>system, medical, health, healthcare</t>
         </is>
       </c>
-      <c r="E82" t="inlineStr"/>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F82" t="inlineStr">
         <is>
           <t>2026-03-10T13:00:04+00:00</t>
@@ -3577,7 +3877,11 @@
           <t>manager, growth, lead, health</t>
         </is>
       </c>
-      <c r="E83" t="inlineStr"/>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F83" t="inlineStr">
         <is>
           <t>2026-03-03T16:00:20+00:00</t>
@@ -3615,7 +3919,11 @@
           <t>manager, design, architect, technical, healthcare, engineering, digital nomad</t>
         </is>
       </c>
-      <c r="E84" t="inlineStr"/>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F84" t="inlineStr">
         <is>
           <t>2026-03-07T00:00:47+00:00</t>
@@ -3655,7 +3963,7 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>18-0</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
@@ -3695,7 +4003,11 @@
           <t>manager, salesforce, travel, cloud, microsoft, management, operational, analytics</t>
         </is>
       </c>
-      <c r="E86" t="inlineStr"/>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F86" t="inlineStr">
         <is>
           <t>2026-03-04T00:01:01+00:00</t>
@@ -3733,7 +4045,11 @@
           <t>saas, software, adult, c, management, senior, marketing, executive, e-commerce</t>
         </is>
       </c>
-      <c r="E87" t="inlineStr"/>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F87" t="inlineStr">
         <is>
           <t>2026-03-03T00:00:21+00:00</t>
@@ -3771,7 +4087,11 @@
           <t>senior</t>
         </is>
       </c>
-      <c r="E88" t="inlineStr"/>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F88" t="inlineStr">
         <is>
           <t>2026-03-03T08:00:29+00:00</t>
@@ -3809,7 +4129,11 @@
           <t>manager, technical, developer, software, lead, senior, digital nomad</t>
         </is>
       </c>
-      <c r="E89" t="inlineStr"/>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F89" t="inlineStr">
         <is>
           <t>2026-03-06T08:00:15+00:00</t>
@@ -3847,7 +4171,11 @@
           <t>software, system, python, engineer, linux</t>
         </is>
       </c>
-      <c r="E90" t="inlineStr"/>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F90" t="inlineStr">
         <is>
           <t>2026-03-03T16:00:31+00:00</t>
@@ -3885,7 +4213,11 @@
           <t>manager, design, saas, crypto, bitcoin, training, technical, software, growth, financial, fintech, cloud, api, leader, management, lead, ops, operations, marketing, engineering, recruitment, executive, digital nomad</t>
         </is>
       </c>
-      <c r="E91" t="inlineStr"/>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F91" t="inlineStr">
         <is>
           <t>2026-03-06T16:00:03+00:00</t>
@@ -3923,7 +4255,11 @@
           <t>ui, ux, designer, support, education</t>
         </is>
       </c>
-      <c r="E92" t="inlineStr"/>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F92" t="inlineStr">
         <is>
           <t>2026-03-05T22:14:41+00:00</t>
@@ -3961,7 +4297,11 @@
           <t>teaching, technical, software, growth, travel, education, management, sales</t>
         </is>
       </c>
-      <c r="E93" t="inlineStr"/>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F93" t="inlineStr">
         <is>
           <t>2026-03-10T16:00:04+00:00</t>
@@ -3999,7 +4339,11 @@
           <t>ios, support</t>
         </is>
       </c>
-      <c r="E94" t="inlineStr"/>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F94" t="inlineStr">
         <is>
           <t>2026-03-05T16:00:07+00:00</t>
@@ -4037,7 +4381,11 @@
           <t>analyst, consultancy, strategy, senior, analytics</t>
         </is>
       </c>
-      <c r="E95" t="inlineStr"/>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F95" t="inlineStr">
         <is>
           <t>2026-03-05T23:00:28+00:00</t>
@@ -4155,7 +4503,11 @@
           <t>manager, support, management</t>
         </is>
       </c>
-      <c r="E98" t="inlineStr"/>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F98" t="inlineStr">
         <is>
           <t>2026-03-07T00:01:10+00:00</t>
@@ -4193,7 +4545,11 @@
           <t>developer, mobile, lead, android, digital nomad</t>
         </is>
       </c>
-      <c r="E99" t="inlineStr"/>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F99" t="inlineStr">
         <is>
           <t>2026-03-06T16:00:11+00:00</t>
@@ -4273,7 +4629,11 @@
           <t>security, design, support, code, management, engineering, digital nomad</t>
         </is>
       </c>
-      <c r="E101" t="inlineStr"/>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="F101" t="inlineStr">
         <is>
           <t>2026-03-10T00:00:06+00:00</t>

</xml_diff>

<commit_message>
harden scraping pipeline, add tests, and refresh README
</commit_message>
<xml_diff>
--- a/output/remote_jobs.xlsx
+++ b/output/remote_jobs.xlsx
@@ -479,11 +479,7 @@
           <t>accountant, support, accounting, payroll, financial, sales, health, healthcare, non tech</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
           <t>2026-03-05T19:00:05+00:00</t>
@@ -521,11 +517,7 @@
           <t>python, game, technical, support, code, math, node, lead</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
           <t>2026-03-09T22:00:13+00:00</t>
@@ -563,11 +555,7 @@
           <t>game, design, designer, mobile, strategy, content, senior, junior, digital nomad</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
           <t>2026-02-28T21:00:14+00:00</t>
@@ -605,11 +593,7 @@
           <t>director, students, training, support, software</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>2026-03-10T06:00:23+00:00</t>
@@ -647,11 +631,7 @@
           <t>architect, design, security, training, technical, growth, serverless, cloud, management, lead, junior, health, engineering, digital nomad</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
           <t>2026-03-03T21:00:19+00:00</t>
@@ -689,11 +669,7 @@
           <t>design, security, training, architect, technical, support, cloud, node, management, operational, health, engineer, digital nomad</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>2026-03-07T20:00:08+00:00</t>
@@ -731,11 +707,7 @@
           <t>design, crypto, security, support, financial, investment, api, lead, operations, operational, digital nomad</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
           <t>2026-03-09T07:00:07+00:00</t>
@@ -773,11 +745,7 @@
           <t>analyst, crypto, training, support, financial, investment, fintech, api, operations, sales, non tech</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
           <t>2026-03-05T11:00:07+00:00</t>
@@ -857,11 +825,7 @@
           <t>manager, technical, software, cloud, operational, engineering</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
           <t>2026-03-07T13:00:12+00:00</t>
@@ -899,11 +863,7 @@
           <t>design, game, technical, developer, animator, animation, content, senior, digital nomad</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
           <t>2026-03-03T21:00:06+00:00</t>
@@ -941,11 +901,7 @@
           <t>assistant, design, support, admin, content, sales, executive, full-time, digital nomad</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
           <t>2026-03-03T07:00:02+00:00</t>
@@ -983,11 +939,7 @@
           <t>support, operational, analytics, engineering</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
           <t>2026-03-07T00:00:35+00:00</t>
@@ -1025,11 +977,7 @@
           <t>developer, back-end, python, reliability, backend, ecommerce, e-commerce, digital nomad</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
           <t>2026-03-06T02:00:12+00:00</t>
@@ -1109,11 +1057,7 @@
           <t>design, designer, growth, web, marketing, go, health, digital nomad</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
           <t>2026-03-10T10:00:06+00:00</t>
@@ -1193,11 +1137,7 @@
           <t>design, system, technical, support, growth, director, lead, senior, engineer, engineering, digital nomad</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr">
         <is>
           <t>2026-03-05T23:00:14+00:00</t>
@@ -1235,11 +1175,7 @@
           <t>manager, web3, security, technical, support, travel, lead, sales, full-time</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr">
         <is>
           <t>2026-03-05T15:00:04+00:00</t>
@@ -1277,11 +1213,7 @@
           <t>teach, technical, support, code, engineer, engineering</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
           <t>2026-03-03T17:00:17+00:00</t>
@@ -1319,11 +1251,7 @@
           <t>design, ansible, security, python, training, support, growth, code, voice, devops, education, banking, mobile, management, senior, sales, go, health, recruiting, engineer, engineering, recruitment, linux, e-commerce, digital nomad</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr">
         <is>
           <t>2026-03-07T00:01:33+00:00</t>
@@ -1361,11 +1289,7 @@
           <t>manager, design, saas, training, support, growth, director, voice, education, banking, mobile, strategy, lead, senior, operations, marketing, sales, go, health, recruiting, recruitment, executive, digital nomad</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr">
         <is>
           <t>2026-03-04T00:01:20+00:00</t>
@@ -1403,11 +1327,7 @@
           <t>security, software, growth, video, analytics</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr">
         <is>
           <t>2026-03-04T00:01:42+00:00</t>
@@ -1445,11 +1365,7 @@
           <t>design, saas, technical, support, growth, strategy, management, operations, operational, digital nomad</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr">
         <is>
           <t>2026-03-09T17:00:06+00:00</t>
@@ -1487,11 +1403,7 @@
           <t>manager, crypto, cryptocurrency, api, operational, marketing, sales</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr">
         <is>
           <t>2026-03-03T18:00:01+00:00</t>
@@ -1529,11 +1441,7 @@
           <t>analyst, embedded, security, training, consultancy, management, senior, executive</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr">
         <is>
           <t>2026-03-04T00:00:42+00:00</t>
@@ -1571,11 +1479,7 @@
           <t>react, software, design, jira, front-end, back-end, security, training, test, code, web, javascript, html, senior, engineer, engineering, digital nomad</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
           <t>2026-03-05T16:00:14+00:00</t>
@@ -1613,11 +1517,7 @@
           <t>support, software, devops, cloud, lead, content, reliability, engineer, engineering</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
           <t>2026-03-07T20:00:19+00:00</t>
@@ -1655,11 +1555,7 @@
           <t>financial, fintech, banking, senior, engineer</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E30" t="inlineStr"/>
       <c r="F30" t="inlineStr">
         <is>
           <t>2026-03-04T08:00:21+00:00</t>
@@ -1739,11 +1635,7 @@
           <t>senior, sales, engineer</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E32" t="inlineStr"/>
       <c r="F32" t="inlineStr">
         <is>
           <t>2026-03-10T00:01:04+00:00</t>
@@ -1781,11 +1673,7 @@
           <t>vfx, technical, lead, engineering</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E33" t="inlineStr"/>
       <c r="F33" t="inlineStr">
         <is>
           <t>2026-03-03T22:00:12+00:00</t>
@@ -1823,11 +1711,7 @@
           <t>unity, designer, senior</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E34" t="inlineStr"/>
       <c r="F34" t="inlineStr">
         <is>
           <t>2026-03-03T22:00:26+00:00</t>
@@ -1865,11 +1749,7 @@
           <t>growth, design, frontend, architect, technical, web, mobile, leader, lead, executive, digital nomad</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E35" t="inlineStr"/>
       <c r="F35" t="inlineStr">
         <is>
           <t>2026-03-04T00:01:31+00:00</t>
@@ -1907,11 +1787,7 @@
           <t>manager, system, technical, software, ui, code, engineering</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E36" t="inlineStr"/>
       <c r="F36" t="inlineStr">
         <is>
           <t>2026-03-03T00:01:09+00:00</t>
@@ -1949,11 +1825,7 @@
           <t>security, design, api, engineer, engineering, digital nomad</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E37" t="inlineStr"/>
       <c r="F37" t="inlineStr">
         <is>
           <t>2026-03-09T08:00:05+00:00</t>
@@ -1991,11 +1863,7 @@
           <t>support, software, senior, engineer, engineering</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E38" t="inlineStr"/>
       <c r="F38" t="inlineStr">
         <is>
           <t>2026-03-03T16:00:17+00:00</t>
@@ -2033,11 +1901,7 @@
           <t>support, financial, finance, fintech, strategy, operations, non tech</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E39" t="inlineStr"/>
       <c r="F39" t="inlineStr">
         <is>
           <t>2026-03-04T00:00:08+00:00</t>
@@ -2075,11 +1939,7 @@
           <t>manager, hr, training, growth, management, lead, senior, operations, reliability</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E40" t="inlineStr"/>
       <c r="F40" t="inlineStr">
         <is>
           <t>2026-03-03T00:00:53+00:00</t>
@@ -2117,11 +1977,7 @@
           <t>python, django, software, design, saas, security, full-stack, technical, developer, testing, code, devops, cloud, git, postgresql, senior, operations, engineer, digital nomad</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E41" t="inlineStr"/>
       <c r="F41" t="inlineStr">
         <is>
           <t>2026-03-09T18:00:23+00:00</t>
@@ -2159,11 +2015,7 @@
           <t>web3, cryptocurrency, voice, lead, content, operations, executive</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E42" t="inlineStr"/>
       <c r="F42" t="inlineStr">
         <is>
           <t>2026-03-09T12:00:02+00:00</t>
@@ -2201,11 +2053,7 @@
           <t>salesforce, technical, support, administrator, management, reliability, health</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E43" t="inlineStr"/>
       <c r="F43" t="inlineStr">
         <is>
           <t>2026-03-03T18:00:12+00:00</t>
@@ -2243,11 +2091,7 @@
           <t>system, teaching, students, technical</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E44" t="inlineStr"/>
       <c r="F44" t="inlineStr">
         <is>
           <t>2026-03-10T00:01:14+00:00</t>
@@ -2285,11 +2129,7 @@
           <t>analyst, support, testing, leader, senior, health, healthcare, non tech</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E45" t="inlineStr"/>
       <c r="F45" t="inlineStr">
         <is>
           <t>2026-03-10T00:00:49+00:00</t>
@@ -2327,11 +2167,7 @@
           <t>design, lead, digital nomad</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E46" t="inlineStr"/>
       <c r="F46" t="inlineStr">
         <is>
           <t>2026-03-10T00:00:18+00:00</t>
@@ -2369,11 +2205,7 @@
           <t>accountant, saas, manager, accounting, financial, go</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E47" t="inlineStr"/>
       <c r="F47" t="inlineStr">
         <is>
           <t>2026-03-05T20:00:07+00:00</t>
@@ -2411,11 +2243,7 @@
           <t>training, support, education, admin, management, content, non tech</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E48" t="inlineStr"/>
       <c r="F48" t="inlineStr">
         <is>
           <t>2026-03-09T08:00:03+00:00</t>
@@ -2449,11 +2277,7 @@
         </is>
       </c>
       <c r="D49" t="inlineStr"/>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E49" t="inlineStr"/>
       <c r="F49" t="inlineStr">
         <is>
           <t>2026-03-04T16:00:04+00:00</t>
@@ -2491,11 +2315,7 @@
           <t>analyst, support, financial, senior, analytics, health, non tech</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E50" t="inlineStr"/>
       <c r="F50" t="inlineStr">
         <is>
           <t>2026-03-07T00:00:56+00:00</t>
@@ -2533,11 +2353,7 @@
           <t>manager, design, system, architect, technical, support, growth, voice, lead, medical, health, engineering, digital nomad</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E51" t="inlineStr"/>
       <c r="F51" t="inlineStr">
         <is>
           <t>2026-03-07T00:00:08+00:00</t>
@@ -2575,11 +2391,7 @@
           <t>manager, design, saas, support, growth, financial, investment, investor, fintech, strategy, management, senior, operational, analytics, sales, reliability, engineering, digital nomad</t>
         </is>
       </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E52" t="inlineStr"/>
       <c r="F52" t="inlineStr">
         <is>
           <t>2026-03-03T00:00:13+00:00</t>
@@ -2617,11 +2429,7 @@
           <t>design, full-stack, architect, testing, operational, engineer, engineering, digital nomad</t>
         </is>
       </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E53" t="inlineStr"/>
       <c r="F53" t="inlineStr">
         <is>
           <t>2026-03-10T00:00:27+00:00</t>
@@ -2659,11 +2467,7 @@
           <t>manager, saas, security, technical, growth, voice, bank, management, lead, android, sales, recruitment, executive</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E54" t="inlineStr"/>
       <c r="F54" t="inlineStr">
         <is>
           <t>2026-03-03T08:00:20+00:00</t>
@@ -2701,11 +2505,7 @@
           <t>manager, copywriting, growth, strategy, management, content, junior</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E55" t="inlineStr"/>
       <c r="F55" t="inlineStr">
         <is>
           <t>2026-03-06T08:00:04+00:00</t>
@@ -2743,11 +2543,7 @@
           <t>full-stack, devops, financial, fintech, cloud, senior, engineer</t>
         </is>
       </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E56" t="inlineStr"/>
       <c r="F56" t="inlineStr">
         <is>
           <t>2026-03-04T00:00:17+00:00</t>
@@ -2827,11 +2623,7 @@
           <t>system, security, software, devops, operations, operational, engineer, linux</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E58" t="inlineStr"/>
       <c r="F58" t="inlineStr">
         <is>
           <t>2026-03-04T17:00:05+00:00</t>
@@ -2869,11 +2661,7 @@
           <t>embedded, growth, analytics, engineer, engineering</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E59" t="inlineStr"/>
       <c r="F59" t="inlineStr">
         <is>
           <t>2026-03-03T16:00:07+00:00</t>
@@ -2911,11 +2699,7 @@
           <t>design, embedded, teach, students, designer, financial, banking, senior, internship, digital nomad</t>
         </is>
       </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E60" t="inlineStr"/>
       <c r="F60" t="inlineStr">
         <is>
           <t>2026-03-03T12:00:05+00:00</t>
@@ -2953,11 +2737,7 @@
           <t>system, coordinator, support, management, operational, medical, health, healthcare</t>
         </is>
       </c>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E61" t="inlineStr"/>
       <c r="F61" t="inlineStr">
         <is>
           <t>2026-03-07T00:00:20+00:00</t>
@@ -2995,11 +2775,7 @@
           <t>training, support, leader, content, health, non tech</t>
         </is>
       </c>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E62" t="inlineStr"/>
       <c r="F62" t="inlineStr">
         <is>
           <t>2026-03-07T00:01:21+00:00</t>
@@ -3037,11 +2813,7 @@
           <t>game, design, designer, technical, lead, content, senior, digital nomad</t>
         </is>
       </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E63" t="inlineStr"/>
       <c r="F63" t="inlineStr">
         <is>
           <t>2026-02-28T21:00:04+00:00</t>
@@ -3079,11 +2851,7 @@
           <t>manager, embedded, growth, director, senior, operational, medical, health</t>
         </is>
       </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E64" t="inlineStr"/>
       <c r="F64" t="inlineStr">
         <is>
           <t>2026-03-10T00:00:42+00:00</t>
@@ -3121,11 +2889,7 @@
           <t>software, design, technical, leader, senior, medical, health, engineer, digital nomad</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E65" t="inlineStr"/>
       <c r="F65" t="inlineStr">
         <is>
           <t>2026-03-10T16:00:07+00:00</t>
@@ -3163,11 +2927,7 @@
           <t>director, training, consult, support, growth, travel, voice, financial, c, leader, strategy, management, lead, senior, marketing, sales, health, recruitment, executive, full-time</t>
         </is>
       </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E66" t="inlineStr"/>
       <c r="F66" t="inlineStr">
         <is>
           <t>2026-03-10T00:00:56+00:00</t>
@@ -3205,11 +2965,7 @@
           <t>director, financial, management, sales</t>
         </is>
       </c>
-      <c r="E67" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E67" t="inlineStr"/>
       <c r="F67" t="inlineStr">
         <is>
           <t>2026-03-03T08:00:13+00:00</t>
@@ -3247,11 +3003,7 @@
           <t>manager, financial, management, sales, non tech</t>
         </is>
       </c>
-      <c r="E68" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E68" t="inlineStr"/>
       <c r="F68" t="inlineStr">
         <is>
           <t>2026-03-04T00:01:12+00:00</t>
@@ -3289,11 +3041,7 @@
           <t>director, saas, system, growth, leader, strategy, lead, sales, medical, health</t>
         </is>
       </c>
-      <c r="E69" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E69" t="inlineStr"/>
       <c r="F69" t="inlineStr">
         <is>
           <t>2026-03-03T00:00:31+00:00</t>
@@ -3331,11 +3079,7 @@
           <t>technical, growth, strategy, lead, senior, health, engineering</t>
         </is>
       </c>
-      <c r="E70" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E70" t="inlineStr"/>
       <c r="F70" t="inlineStr">
         <is>
           <t>2026-03-09T18:00:06+00:00</t>
@@ -3373,11 +3117,7 @@
           <t>software, react, front-end, technical, code, mobile, leader, health, healthcare, engineer, engineering</t>
         </is>
       </c>
-      <c r="E71" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E71" t="inlineStr"/>
       <c r="F71" t="inlineStr">
         <is>
           <t>2026-03-04T00:00:29+00:00</t>
@@ -3415,11 +3155,7 @@
           <t>frontend, design, software, growth, web, management, engineer, backend, digital nomad</t>
         </is>
       </c>
-      <c r="E72" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E72" t="inlineStr"/>
       <c r="F72" t="inlineStr">
         <is>
           <t>2026-03-09T09:00:04+00:00</t>
@@ -3457,11 +3193,7 @@
           <t>support, content</t>
         </is>
       </c>
-      <c r="E73" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E73" t="inlineStr"/>
       <c r="F73" t="inlineStr">
         <is>
           <t>2026-03-03T18:00:40+00:00</t>
@@ -3499,11 +3231,7 @@
           <t>support, content</t>
         </is>
       </c>
-      <c r="E74" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E74" t="inlineStr"/>
       <c r="F74" t="inlineStr">
         <is>
           <t>2026-03-03T18:00:21+00:00</t>
@@ -3541,11 +3269,7 @@
           <t>growth, marketing, analytics, sales, executive</t>
         </is>
       </c>
-      <c r="E75" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E75" t="inlineStr"/>
       <c r="F75" t="inlineStr">
         <is>
           <t>2026-03-03T00:00:06+00:00</t>
@@ -3625,11 +3349,7 @@
           <t>training, technical, testing, test, code, travel, microsoft, senior, legal, health</t>
         </is>
       </c>
-      <c r="E77" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E77" t="inlineStr"/>
       <c r="F77" t="inlineStr">
         <is>
           <t>2026-03-10T08:00:17+00:00</t>
@@ -3667,11 +3387,7 @@
           <t>full-stack, technical, support, growth, code, cloud, management, operational, sales, engineer, engineering</t>
         </is>
       </c>
-      <c r="E78" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E78" t="inlineStr"/>
       <c r="F78" t="inlineStr">
         <is>
           <t>2026-03-06T07:00:06+00:00</t>
@@ -3709,11 +3425,7 @@
           <t>python, technical, support, financial, fintech, analytics, go, health, engineering</t>
         </is>
       </c>
-      <c r="E79" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E79" t="inlineStr"/>
       <c r="F79" t="inlineStr">
         <is>
           <t>2026-03-10T08:00:11+00:00</t>
@@ -3751,11 +3463,7 @@
           <t>manager, support, operations, operational</t>
         </is>
       </c>
-      <c r="E80" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E80" t="inlineStr"/>
       <c r="F80" t="inlineStr">
         <is>
           <t>2026-03-10T09:00:06+00:00</t>
@@ -3793,11 +3501,7 @@
           <t>system, technical, operations, operational</t>
         </is>
       </c>
-      <c r="E81" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E81" t="inlineStr"/>
       <c r="F81" t="inlineStr">
         <is>
           <t>2026-03-03T08:00:03+00:00</t>
@@ -3835,11 +3539,7 @@
           <t>system, medical, health, healthcare</t>
         </is>
       </c>
-      <c r="E82" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E82" t="inlineStr"/>
       <c r="F82" t="inlineStr">
         <is>
           <t>2026-03-10T13:00:04+00:00</t>
@@ -3877,11 +3577,7 @@
           <t>manager, growth, lead, health</t>
         </is>
       </c>
-      <c r="E83" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E83" t="inlineStr"/>
       <c r="F83" t="inlineStr">
         <is>
           <t>2026-03-03T16:00:20+00:00</t>
@@ -3919,11 +3615,7 @@
           <t>manager, design, architect, technical, healthcare, engineering, digital nomad</t>
         </is>
       </c>
-      <c r="E84" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E84" t="inlineStr"/>
       <c r="F84" t="inlineStr">
         <is>
           <t>2026-03-07T00:00:47+00:00</t>
@@ -4003,11 +3695,7 @@
           <t>manager, salesforce, travel, cloud, microsoft, management, operational, analytics</t>
         </is>
       </c>
-      <c r="E86" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E86" t="inlineStr"/>
       <c r="F86" t="inlineStr">
         <is>
           <t>2026-03-04T00:01:01+00:00</t>
@@ -4045,11 +3733,7 @@
           <t>saas, software, adult, c, management, senior, marketing, executive, e-commerce</t>
         </is>
       </c>
-      <c r="E87" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E87" t="inlineStr"/>
       <c r="F87" t="inlineStr">
         <is>
           <t>2026-03-03T00:00:21+00:00</t>
@@ -4087,11 +3771,7 @@
           <t>senior</t>
         </is>
       </c>
-      <c r="E88" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E88" t="inlineStr"/>
       <c r="F88" t="inlineStr">
         <is>
           <t>2026-03-03T08:00:29+00:00</t>
@@ -4129,11 +3809,7 @@
           <t>manager, technical, developer, software, lead, senior, digital nomad</t>
         </is>
       </c>
-      <c r="E89" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E89" t="inlineStr"/>
       <c r="F89" t="inlineStr">
         <is>
           <t>2026-03-06T08:00:15+00:00</t>
@@ -4171,11 +3847,7 @@
           <t>software, system, python, engineer, linux</t>
         </is>
       </c>
-      <c r="E90" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E90" t="inlineStr"/>
       <c r="F90" t="inlineStr">
         <is>
           <t>2026-03-03T16:00:31+00:00</t>
@@ -4213,11 +3885,7 @@
           <t>manager, design, saas, crypto, bitcoin, training, technical, software, growth, financial, fintech, cloud, api, leader, management, lead, ops, operations, marketing, engineering, recruitment, executive, digital nomad</t>
         </is>
       </c>
-      <c r="E91" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E91" t="inlineStr"/>
       <c r="F91" t="inlineStr">
         <is>
           <t>2026-03-06T16:00:03+00:00</t>
@@ -4255,11 +3923,7 @@
           <t>ui, ux, designer, support, education</t>
         </is>
       </c>
-      <c r="E92" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E92" t="inlineStr"/>
       <c r="F92" t="inlineStr">
         <is>
           <t>2026-03-05T22:14:41+00:00</t>
@@ -4297,11 +3961,7 @@
           <t>teaching, technical, software, growth, travel, education, management, sales</t>
         </is>
       </c>
-      <c r="E93" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E93" t="inlineStr"/>
       <c r="F93" t="inlineStr">
         <is>
           <t>2026-03-10T16:00:04+00:00</t>
@@ -4339,11 +3999,7 @@
           <t>ios, support</t>
         </is>
       </c>
-      <c r="E94" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E94" t="inlineStr"/>
       <c r="F94" t="inlineStr">
         <is>
           <t>2026-03-05T16:00:07+00:00</t>
@@ -4381,11 +4037,7 @@
           <t>analyst, consultancy, strategy, senior, analytics</t>
         </is>
       </c>
-      <c r="E95" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E95" t="inlineStr"/>
       <c r="F95" t="inlineStr">
         <is>
           <t>2026-03-05T23:00:28+00:00</t>
@@ -4503,11 +4155,7 @@
           <t>manager, support, management</t>
         </is>
       </c>
-      <c r="E98" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E98" t="inlineStr"/>
       <c r="F98" t="inlineStr">
         <is>
           <t>2026-03-07T00:01:10+00:00</t>
@@ -4545,11 +4193,7 @@
           <t>developer, mobile, lead, android, digital nomad</t>
         </is>
       </c>
-      <c r="E99" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E99" t="inlineStr"/>
       <c r="F99" t="inlineStr">
         <is>
           <t>2026-03-06T16:00:11+00:00</t>
@@ -4629,11 +4273,7 @@
           <t>security, design, support, code, management, engineering, digital nomad</t>
         </is>
       </c>
-      <c r="E101" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="E101" t="inlineStr"/>
       <c r="F101" t="inlineStr">
         <is>
           <t>2026-03-10T00:00:06+00:00</t>

</xml_diff>